<commit_message>
fix: thêm report tổng hợp
</commit_message>
<xml_diff>
--- a/udpate.xlsx
+++ b/udpate.xlsx
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>CD01</t>
   </si>
@@ -223,7 +223,10 @@
     <t>CD63</t>
   </si>
   <si>
-    <t>17B</t>
+    <t>BT1</t>
+  </si>
+  <si>
+    <t>17A</t>
   </si>
 </sst>
 </file>
@@ -930,7 +933,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -957,14 +960,8 @@
     <xf numFmtId="178" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1751,24 +1748,12 @@
       <c r="BB1" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="BC1" s="7">
-        <v>70</v>
-      </c>
-      <c r="BD1" s="7">
-        <v>71</v>
-      </c>
-      <c r="BE1" s="7">
-        <v>72</v>
-      </c>
-      <c r="BF1" s="7">
-        <v>73</v>
-      </c>
-      <c r="BG1" s="7">
-        <v>74</v>
-      </c>
-      <c r="BH1" s="7">
-        <v>75</v>
-      </c>
+      <c r="BC1" s="7"/>
+      <c r="BD1" s="7"/>
+      <c r="BE1" s="7"/>
+      <c r="BF1" s="7"/>
+      <c r="BG1" s="7"/>
+      <c r="BH1" s="7"/>
     </row>
     <row r="2" s="2" customFormat="1" spans="1:60">
       <c r="A2" s="8" t="s">
@@ -1872,94 +1857,167 @@
         <f>204-50</f>
         <v>154</v>
       </c>
-      <c r="AS2" s="15">
+      <c r="AS2" s="13">
         <v>2700</v>
       </c>
-      <c r="AT2" s="15">
+      <c r="AT2" s="13">
         <v>1500</v>
       </c>
-      <c r="AU2" s="15">
+      <c r="AU2" s="13">
         <v>1200</v>
       </c>
-      <c r="AV2" s="15">
+      <c r="AV2" s="13">
         <v>985</v>
       </c>
-      <c r="AW2" s="15">
+      <c r="AW2" s="13">
         <v>1200</v>
       </c>
-      <c r="AX2" s="15">
+      <c r="AX2" s="13">
         <v>1000</v>
       </c>
-      <c r="AY2" s="15">
+      <c r="AY2" s="13">
         <v>615</v>
       </c>
-      <c r="AZ2" s="15"/>
-      <c r="BA2" s="15"/>
-      <c r="BB2" s="15">
+      <c r="AZ2" s="13"/>
+      <c r="BA2" s="13"/>
+      <c r="BB2" s="13">
         <v>2000</v>
       </c>
-      <c r="BC2" s="15"/>
-      <c r="BD2" s="15"/>
-      <c r="BE2" s="15"/>
-      <c r="BF2" s="15"/>
-      <c r="BG2" s="15"/>
+      <c r="BC2" s="13"/>
+      <c r="BD2" s="13"/>
+      <c r="BE2" s="13"/>
+      <c r="BF2" s="13"/>
+      <c r="BG2" s="13"/>
       <c r="BH2" s="9"/>
     </row>
     <row r="3" s="2" customFormat="1" spans="1:60">
-      <c r="A3" s="10"/>
-      <c r="B3" s="9"/>
+      <c r="A3" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="9">
+        <v>2301</v>
+      </c>
       <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
+      <c r="D3" s="9">
+        <v>4001</v>
+      </c>
       <c r="E3" s="9"/>
       <c r="F3" s="9"/>
       <c r="G3" s="9"/>
       <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
+      <c r="I3" s="9">
+        <v>2501</v>
+      </c>
+      <c r="J3" s="9">
+        <v>4501</v>
+      </c>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="9"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
+      <c r="N3" s="9">
+        <v>1401</v>
+      </c>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9">
+        <v>1401</v>
+      </c>
+      <c r="Q3" s="9"/>
       <c r="R3" s="9"/>
       <c r="S3" s="9"/>
       <c r="T3" s="9"/>
       <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
+      <c r="V3" s="9">
+        <v>4601</v>
+      </c>
       <c r="W3" s="9"/>
-      <c r="X3" s="9"/>
-      <c r="Y3" s="9"/>
-      <c r="Z3" s="9"/>
+      <c r="X3" s="9" t="e">
+        <f>'[1]ĐG- XƯỞNG 1'!AA6*2</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Y3" s="9" t="e">
+        <f>'[1]ĐG- XƯỞNG 1'!AB6*2</f>
+        <v>#REF!</v>
+      </c>
+      <c r="Z3" s="9" t="e">
+        <f>'[1]ĐG- XƯỞNG 1'!AC6+200</f>
+        <v>#REF!</v>
+      </c>
       <c r="AA3" s="9"/>
       <c r="AB3" s="9"/>
       <c r="AC3" s="9"/>
       <c r="AD3" s="9"/>
-      <c r="AE3" s="9"/>
-      <c r="AF3" s="9"/>
-      <c r="AG3" s="9"/>
-      <c r="AH3" s="9"/>
-      <c r="AI3" s="9"/>
-      <c r="AJ3" s="9"/>
+      <c r="AE3" s="9">
+        <v>2501</v>
+      </c>
+      <c r="AF3" s="9">
+        <v>1001</v>
+      </c>
+      <c r="AG3" s="9">
+        <v>16</v>
+      </c>
+      <c r="AH3" s="9">
+        <v>1001</v>
+      </c>
+      <c r="AI3" s="9">
+        <v>17</v>
+      </c>
+      <c r="AJ3" s="9">
+        <v>1801</v>
+      </c>
       <c r="AK3" s="9"/>
-      <c r="AL3" s="9"/>
-      <c r="AM3" s="9"/>
-      <c r="AN3" s="9"/>
-      <c r="AO3" s="9"/>
-      <c r="AP3" s="9"/>
-      <c r="AQ3" s="9"/>
-      <c r="AR3" s="9"/>
-      <c r="AS3" s="9"/>
-      <c r="AT3" s="9"/>
-      <c r="AU3" s="9"/>
-      <c r="AV3" s="9"/>
-      <c r="AW3" s="9"/>
-      <c r="AX3" s="9"/>
-      <c r="AY3" s="9"/>
-      <c r="AZ3" s="9"/>
-      <c r="BA3" s="9"/>
-      <c r="BB3" s="9"/>
+      <c r="AL3" s="9">
+        <v>1301</v>
+      </c>
+      <c r="AM3" s="9">
+        <f>471-50+88</f>
+        <v>509</v>
+      </c>
+      <c r="AN3" s="9">
+        <f>311-50</f>
+        <v>261</v>
+      </c>
+      <c r="AO3" s="9">
+        <f>311-50</f>
+        <v>261</v>
+      </c>
+      <c r="AP3" s="9">
+        <f>311-50</f>
+        <v>261</v>
+      </c>
+      <c r="AQ3" s="9">
+        <f>204-50</f>
+        <v>154</v>
+      </c>
+      <c r="AR3" s="9">
+        <f>204-50</f>
+        <v>154</v>
+      </c>
+      <c r="AS3" s="13">
+        <v>2701</v>
+      </c>
+      <c r="AT3" s="13">
+        <v>1501</v>
+      </c>
+      <c r="AU3" s="13">
+        <v>1201</v>
+      </c>
+      <c r="AV3" s="13">
+        <v>986</v>
+      </c>
+      <c r="AW3" s="13">
+        <v>1201</v>
+      </c>
+      <c r="AX3" s="13">
+        <v>1001</v>
+      </c>
+      <c r="AY3" s="13">
+        <v>616</v>
+      </c>
+      <c r="AZ3" s="13"/>
+      <c r="BA3" s="13"/>
+      <c r="BB3" s="13">
+        <v>2001</v>
+      </c>
       <c r="BC3" s="9"/>
       <c r="BD3" s="9"/>
       <c r="BE3" s="9"/>
@@ -1968,492 +2026,492 @@
       <c r="BH3" s="9"/>
     </row>
     <row r="4" s="3" customFormat="1" spans="2:60">
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="14"/>
-      <c r="P4" s="14"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="14"/>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="14"/>
-      <c r="AB4" s="14"/>
-      <c r="AC4" s="14"/>
-      <c r="AD4" s="14"/>
-      <c r="AE4" s="14"/>
-      <c r="AF4" s="14"/>
-      <c r="AG4" s="14"/>
-      <c r="AH4" s="14"/>
-      <c r="AI4" s="14"/>
-      <c r="AJ4" s="14"/>
-      <c r="AK4" s="14"/>
-      <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
-      <c r="AN4" s="14"/>
-      <c r="AO4" s="14"/>
-      <c r="AP4" s="14"/>
-      <c r="AQ4" s="14"/>
-      <c r="AR4" s="14"/>
-      <c r="AS4" s="14"/>
-      <c r="AT4" s="14"/>
-      <c r="AU4" s="14"/>
-      <c r="AV4" s="14"/>
-      <c r="AW4" s="14"/>
-      <c r="AX4" s="14"/>
-      <c r="AY4" s="14"/>
-      <c r="AZ4" s="14"/>
-      <c r="BA4" s="14"/>
-      <c r="BB4" s="14"/>
-      <c r="BC4" s="14"/>
-      <c r="BD4" s="14"/>
-      <c r="BE4" s="14"/>
-      <c r="BF4" s="14"/>
-      <c r="BG4" s="14"/>
-      <c r="BH4" s="14"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
+      <c r="AB4" s="12"/>
+      <c r="AC4" s="12"/>
+      <c r="AD4" s="12"/>
+      <c r="AE4" s="12"/>
+      <c r="AF4" s="12"/>
+      <c r="AG4" s="12"/>
+      <c r="AH4" s="12"/>
+      <c r="AI4" s="12"/>
+      <c r="AJ4" s="12"/>
+      <c r="AK4" s="12"/>
+      <c r="AL4" s="12"/>
+      <c r="AM4" s="12"/>
+      <c r="AN4" s="12"/>
+      <c r="AO4" s="12"/>
+      <c r="AP4" s="12"/>
+      <c r="AQ4" s="12"/>
+      <c r="AR4" s="12"/>
+      <c r="AS4" s="12"/>
+      <c r="AT4" s="12"/>
+      <c r="AU4" s="12"/>
+      <c r="AV4" s="12"/>
+      <c r="AW4" s="12"/>
+      <c r="AX4" s="12"/>
+      <c r="AY4" s="12"/>
+      <c r="AZ4" s="12"/>
+      <c r="BA4" s="12"/>
+      <c r="BB4" s="12"/>
+      <c r="BC4" s="12"/>
+      <c r="BD4" s="12"/>
+      <c r="BE4" s="12"/>
+      <c r="BF4" s="12"/>
+      <c r="BG4" s="12"/>
+      <c r="BH4" s="12"/>
     </row>
     <row r="5" s="3" customFormat="1" spans="2:60">
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="14"/>
-      <c r="T5" s="14"/>
-      <c r="U5" s="14"/>
-      <c r="V5" s="14"/>
-      <c r="W5" s="14"/>
-      <c r="X5" s="14"/>
-      <c r="Y5" s="14"/>
-      <c r="Z5" s="14"/>
-      <c r="AA5" s="14"/>
-      <c r="AB5" s="14"/>
-      <c r="AC5" s="14"/>
-      <c r="AD5" s="14"/>
-      <c r="AE5" s="14"/>
-      <c r="AF5" s="14"/>
-      <c r="AG5" s="14"/>
-      <c r="AH5" s="14"/>
-      <c r="AI5" s="14"/>
-      <c r="AJ5" s="14"/>
-      <c r="AK5" s="14"/>
-      <c r="AL5" s="14"/>
-      <c r="AM5" s="14"/>
-      <c r="AN5" s="14"/>
-      <c r="AO5" s="14"/>
-      <c r="AP5" s="14"/>
-      <c r="AQ5" s="14"/>
-      <c r="AR5" s="14"/>
-      <c r="AS5" s="14"/>
-      <c r="AT5" s="14"/>
-      <c r="AU5" s="14"/>
-      <c r="AV5" s="14"/>
-      <c r="AW5" s="14"/>
-      <c r="AX5" s="14"/>
-      <c r="AY5" s="14"/>
-      <c r="AZ5" s="14"/>
-      <c r="BA5" s="14"/>
-      <c r="BB5" s="14"/>
-      <c r="BC5" s="14"/>
-      <c r="BD5" s="14"/>
-      <c r="BE5" s="14"/>
-      <c r="BF5" s="14"/>
-      <c r="BG5" s="14"/>
-      <c r="BH5" s="14"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
+      <c r="U5" s="12"/>
+      <c r="V5" s="12"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="12"/>
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="12"/>
+      <c r="AA5" s="12"/>
+      <c r="AB5" s="12"/>
+      <c r="AC5" s="12"/>
+      <c r="AD5" s="12"/>
+      <c r="AE5" s="12"/>
+      <c r="AF5" s="12"/>
+      <c r="AG5" s="12"/>
+      <c r="AH5" s="12"/>
+      <c r="AI5" s="12"/>
+      <c r="AJ5" s="12"/>
+      <c r="AK5" s="12"/>
+      <c r="AL5" s="12"/>
+      <c r="AM5" s="12"/>
+      <c r="AN5" s="12"/>
+      <c r="AO5" s="12"/>
+      <c r="AP5" s="12"/>
+      <c r="AQ5" s="12"/>
+      <c r="AR5" s="12"/>
+      <c r="AS5" s="12"/>
+      <c r="AT5" s="12"/>
+      <c r="AU5" s="12"/>
+      <c r="AV5" s="12"/>
+      <c r="AW5" s="12"/>
+      <c r="AX5" s="12"/>
+      <c r="AY5" s="12"/>
+      <c r="AZ5" s="12"/>
+      <c r="BA5" s="12"/>
+      <c r="BB5" s="12"/>
+      <c r="BC5" s="12"/>
+      <c r="BD5" s="12"/>
+      <c r="BE5" s="12"/>
+      <c r="BF5" s="12"/>
+      <c r="BG5" s="12"/>
+      <c r="BH5" s="12"/>
     </row>
     <row r="6" s="3" customFormat="1" spans="2:60">
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="14"/>
-      <c r="S6" s="14"/>
-      <c r="T6" s="14"/>
-      <c r="U6" s="14"/>
-      <c r="V6" s="14"/>
-      <c r="W6" s="14"/>
-      <c r="X6" s="14"/>
-      <c r="Y6" s="14"/>
-      <c r="Z6" s="14"/>
-      <c r="AA6" s="14"/>
-      <c r="AB6" s="14"/>
-      <c r="AC6" s="14"/>
-      <c r="AD6" s="14"/>
-      <c r="AE6" s="14"/>
-      <c r="AF6" s="14"/>
-      <c r="AG6" s="14"/>
-      <c r="AH6" s="14"/>
-      <c r="AI6" s="14"/>
-      <c r="AJ6" s="14"/>
-      <c r="AK6" s="14"/>
-      <c r="AL6" s="14"/>
-      <c r="AM6" s="14"/>
-      <c r="AN6" s="14"/>
-      <c r="AO6" s="14"/>
-      <c r="AP6" s="14"/>
-      <c r="AQ6" s="14"/>
-      <c r="AR6" s="14"/>
-      <c r="AS6" s="14"/>
-      <c r="AT6" s="14"/>
-      <c r="AU6" s="14"/>
-      <c r="AV6" s="14"/>
-      <c r="AW6" s="14"/>
-      <c r="AX6" s="14"/>
-      <c r="AY6" s="14"/>
-      <c r="AZ6" s="14"/>
-      <c r="BA6" s="14"/>
-      <c r="BB6" s="14"/>
-      <c r="BC6" s="14"/>
-      <c r="BD6" s="14"/>
-      <c r="BE6" s="14"/>
-      <c r="BF6" s="14"/>
-      <c r="BG6" s="14"/>
-      <c r="BH6" s="14"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="12"/>
+      <c r="W6" s="12"/>
+      <c r="X6" s="12"/>
+      <c r="Y6" s="12"/>
+      <c r="Z6" s="12"/>
+      <c r="AA6" s="12"/>
+      <c r="AB6" s="12"/>
+      <c r="AC6" s="12"/>
+      <c r="AD6" s="12"/>
+      <c r="AE6" s="12"/>
+      <c r="AF6" s="12"/>
+      <c r="AG6" s="12"/>
+      <c r="AH6" s="12"/>
+      <c r="AI6" s="12"/>
+      <c r="AJ6" s="12"/>
+      <c r="AK6" s="12"/>
+      <c r="AL6" s="12"/>
+      <c r="AM6" s="12"/>
+      <c r="AN6" s="12"/>
+      <c r="AO6" s="12"/>
+      <c r="AP6" s="12"/>
+      <c r="AQ6" s="12"/>
+      <c r="AR6" s="12"/>
+      <c r="AS6" s="12"/>
+      <c r="AT6" s="12"/>
+      <c r="AU6" s="12"/>
+      <c r="AV6" s="12"/>
+      <c r="AW6" s="12"/>
+      <c r="AX6" s="12"/>
+      <c r="AY6" s="12"/>
+      <c r="AZ6" s="12"/>
+      <c r="BA6" s="12"/>
+      <c r="BB6" s="12"/>
+      <c r="BC6" s="12"/>
+      <c r="BD6" s="12"/>
+      <c r="BE6" s="12"/>
+      <c r="BF6" s="12"/>
+      <c r="BG6" s="12"/>
+      <c r="BH6" s="12"/>
     </row>
     <row r="7" s="3" customFormat="1" spans="2:60">
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="14"/>
-      <c r="Q7" s="14"/>
-      <c r="R7" s="14"/>
-      <c r="S7" s="14"/>
-      <c r="T7" s="14"/>
-      <c r="U7" s="14"/>
-      <c r="V7" s="14"/>
-      <c r="W7" s="14"/>
-      <c r="X7" s="14"/>
-      <c r="Y7" s="14"/>
-      <c r="Z7" s="14"/>
-      <c r="AA7" s="14"/>
-      <c r="AB7" s="14"/>
-      <c r="AC7" s="14"/>
-      <c r="AD7" s="14"/>
-      <c r="AE7" s="14"/>
-      <c r="AF7" s="14"/>
-      <c r="AG7" s="14"/>
-      <c r="AH7" s="14"/>
-      <c r="AI7" s="14"/>
-      <c r="AJ7" s="14"/>
-      <c r="AK7" s="14"/>
-      <c r="AL7" s="14"/>
-      <c r="AM7" s="14"/>
-      <c r="AN7" s="14"/>
-      <c r="AO7" s="14"/>
-      <c r="AP7" s="14"/>
-      <c r="AQ7" s="14"/>
-      <c r="AR7" s="14"/>
-      <c r="AS7" s="14"/>
-      <c r="AT7" s="14"/>
-      <c r="AU7" s="14"/>
-      <c r="AV7" s="14"/>
-      <c r="AW7" s="14"/>
-      <c r="AX7" s="14"/>
-      <c r="AY7" s="14"/>
-      <c r="AZ7" s="14"/>
-      <c r="BA7" s="14"/>
-      <c r="BB7" s="14"/>
-      <c r="BC7" s="14"/>
-      <c r="BD7" s="14"/>
-      <c r="BE7" s="14"/>
-      <c r="BF7" s="14"/>
-      <c r="BG7" s="14"/>
-      <c r="BH7" s="14"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="12"/>
+      <c r="T7" s="12"/>
+      <c r="U7" s="12"/>
+      <c r="V7" s="12"/>
+      <c r="W7" s="12"/>
+      <c r="X7" s="12"/>
+      <c r="Y7" s="12"/>
+      <c r="Z7" s="12"/>
+      <c r="AA7" s="12"/>
+      <c r="AB7" s="12"/>
+      <c r="AC7" s="12"/>
+      <c r="AD7" s="12"/>
+      <c r="AE7" s="12"/>
+      <c r="AF7" s="12"/>
+      <c r="AG7" s="12"/>
+      <c r="AH7" s="12"/>
+      <c r="AI7" s="12"/>
+      <c r="AJ7" s="12"/>
+      <c r="AK7" s="12"/>
+      <c r="AL7" s="12"/>
+      <c r="AM7" s="12"/>
+      <c r="AN7" s="12"/>
+      <c r="AO7" s="12"/>
+      <c r="AP7" s="12"/>
+      <c r="AQ7" s="12"/>
+      <c r="AR7" s="12"/>
+      <c r="AS7" s="12"/>
+      <c r="AT7" s="12"/>
+      <c r="AU7" s="12"/>
+      <c r="AV7" s="12"/>
+      <c r="AW7" s="12"/>
+      <c r="AX7" s="12"/>
+      <c r="AY7" s="12"/>
+      <c r="AZ7" s="12"/>
+      <c r="BA7" s="12"/>
+      <c r="BB7" s="12"/>
+      <c r="BC7" s="12"/>
+      <c r="BD7" s="12"/>
+      <c r="BE7" s="12"/>
+      <c r="BF7" s="12"/>
+      <c r="BG7" s="12"/>
+      <c r="BH7" s="12"/>
     </row>
     <row r="8" s="3" customFormat="1" spans="2:60">
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
-      <c r="U8" s="14"/>
-      <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="14"/>
-      <c r="Y8" s="14"/>
-      <c r="Z8" s="14"/>
-      <c r="AA8" s="14"/>
-      <c r="AB8" s="14"/>
-      <c r="AC8" s="14"/>
-      <c r="AD8" s="14"/>
-      <c r="AE8" s="14"/>
-      <c r="AF8" s="14"/>
-      <c r="AG8" s="14"/>
-      <c r="AH8" s="14"/>
-      <c r="AI8" s="14"/>
-      <c r="AJ8" s="14"/>
-      <c r="AK8" s="14"/>
-      <c r="AL8" s="14"/>
-      <c r="AM8" s="14"/>
-      <c r="AN8" s="14"/>
-      <c r="AO8" s="14"/>
-      <c r="AP8" s="14"/>
-      <c r="AQ8" s="14"/>
-      <c r="AR8" s="14"/>
-      <c r="AS8" s="14"/>
-      <c r="AT8" s="14"/>
-      <c r="AU8" s="14"/>
-      <c r="AV8" s="14"/>
-      <c r="AW8" s="14"/>
-      <c r="AX8" s="14"/>
-      <c r="AY8" s="14"/>
-      <c r="AZ8" s="14"/>
-      <c r="BA8" s="14"/>
-      <c r="BB8" s="14"/>
-      <c r="BC8" s="14"/>
-      <c r="BD8" s="14"/>
-      <c r="BE8" s="14"/>
-      <c r="BF8" s="14"/>
-      <c r="BG8" s="14"/>
-      <c r="BH8" s="14"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="12"/>
+      <c r="W8" s="12"/>
+      <c r="X8" s="12"/>
+      <c r="Y8" s="12"/>
+      <c r="Z8" s="12"/>
+      <c r="AA8" s="12"/>
+      <c r="AB8" s="12"/>
+      <c r="AC8" s="12"/>
+      <c r="AD8" s="12"/>
+      <c r="AE8" s="12"/>
+      <c r="AF8" s="12"/>
+      <c r="AG8" s="12"/>
+      <c r="AH8" s="12"/>
+      <c r="AI8" s="12"/>
+      <c r="AJ8" s="12"/>
+      <c r="AK8" s="12"/>
+      <c r="AL8" s="12"/>
+      <c r="AM8" s="12"/>
+      <c r="AN8" s="12"/>
+      <c r="AO8" s="12"/>
+      <c r="AP8" s="12"/>
+      <c r="AQ8" s="12"/>
+      <c r="AR8" s="12"/>
+      <c r="AS8" s="12"/>
+      <c r="AT8" s="12"/>
+      <c r="AU8" s="12"/>
+      <c r="AV8" s="12"/>
+      <c r="AW8" s="12"/>
+      <c r="AX8" s="12"/>
+      <c r="AY8" s="12"/>
+      <c r="AZ8" s="12"/>
+      <c r="BA8" s="12"/>
+      <c r="BB8" s="12"/>
+      <c r="BC8" s="12"/>
+      <c r="BD8" s="12"/>
+      <c r="BE8" s="12"/>
+      <c r="BF8" s="12"/>
+      <c r="BG8" s="12"/>
+      <c r="BH8" s="12"/>
     </row>
     <row r="9" s="3" customFormat="1" spans="2:60">
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="14"/>
-      <c r="O9" s="14"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="14"/>
-      <c r="R9" s="14"/>
-      <c r="S9" s="14"/>
-      <c r="T9" s="14"/>
-      <c r="U9" s="14"/>
-      <c r="V9" s="14"/>
-      <c r="W9" s="14"/>
-      <c r="X9" s="14"/>
-      <c r="Y9" s="14"/>
-      <c r="Z9" s="14"/>
-      <c r="AA9" s="14"/>
-      <c r="AB9" s="14"/>
-      <c r="AC9" s="14"/>
-      <c r="AD9" s="14"/>
-      <c r="AE9" s="14"/>
-      <c r="AF9" s="14"/>
-      <c r="AG9" s="14"/>
-      <c r="AH9" s="14"/>
-      <c r="AI9" s="14"/>
-      <c r="AJ9" s="14"/>
-      <c r="AK9" s="14"/>
-      <c r="AL9" s="14"/>
-      <c r="AM9" s="14"/>
-      <c r="AN9" s="14"/>
-      <c r="AO9" s="14"/>
-      <c r="AP9" s="14"/>
-      <c r="AQ9" s="14"/>
-      <c r="AR9" s="14"/>
-      <c r="AS9" s="14"/>
-      <c r="AT9" s="14"/>
-      <c r="AU9" s="14"/>
-      <c r="AV9" s="14"/>
-      <c r="AW9" s="14"/>
-      <c r="AX9" s="14"/>
-      <c r="AY9" s="14"/>
-      <c r="AZ9" s="14"/>
-      <c r="BA9" s="14"/>
-      <c r="BB9" s="14"/>
-      <c r="BC9" s="14"/>
-      <c r="BD9" s="14"/>
-      <c r="BE9" s="14"/>
-      <c r="BF9" s="14"/>
-      <c r="BG9" s="14"/>
-      <c r="BH9" s="14"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="12"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="12"/>
+      <c r="Y9" s="12"/>
+      <c r="Z9" s="12"/>
+      <c r="AA9" s="12"/>
+      <c r="AB9" s="12"/>
+      <c r="AC9" s="12"/>
+      <c r="AD9" s="12"/>
+      <c r="AE9" s="12"/>
+      <c r="AF9" s="12"/>
+      <c r="AG9" s="12"/>
+      <c r="AH9" s="12"/>
+      <c r="AI9" s="12"/>
+      <c r="AJ9" s="12"/>
+      <c r="AK9" s="12"/>
+      <c r="AL9" s="12"/>
+      <c r="AM9" s="12"/>
+      <c r="AN9" s="12"/>
+      <c r="AO9" s="12"/>
+      <c r="AP9" s="12"/>
+      <c r="AQ9" s="12"/>
+      <c r="AR9" s="12"/>
+      <c r="AS9" s="12"/>
+      <c r="AT9" s="12"/>
+      <c r="AU9" s="12"/>
+      <c r="AV9" s="12"/>
+      <c r="AW9" s="12"/>
+      <c r="AX9" s="12"/>
+      <c r="AY9" s="12"/>
+      <c r="AZ9" s="12"/>
+      <c r="BA9" s="12"/>
+      <c r="BB9" s="12"/>
+      <c r="BC9" s="12"/>
+      <c r="BD9" s="12"/>
+      <c r="BE9" s="12"/>
+      <c r="BF9" s="12"/>
+      <c r="BG9" s="12"/>
+      <c r="BH9" s="12"/>
     </row>
     <row r="10" s="3" customFormat="1" spans="2:60">
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
-      <c r="R10" s="14"/>
-      <c r="S10" s="14"/>
-      <c r="T10" s="14"/>
-      <c r="U10" s="14"/>
-      <c r="V10" s="14"/>
-      <c r="W10" s="14"/>
-      <c r="X10" s="14"/>
-      <c r="Y10" s="14"/>
-      <c r="Z10" s="14"/>
-      <c r="AA10" s="14"/>
-      <c r="AB10" s="14"/>
-      <c r="AC10" s="14"/>
-      <c r="AD10" s="14"/>
-      <c r="AE10" s="14"/>
-      <c r="AF10" s="14"/>
-      <c r="AG10" s="14"/>
-      <c r="AH10" s="14"/>
-      <c r="AI10" s="14"/>
-      <c r="AJ10" s="14"/>
-      <c r="AK10" s="14"/>
-      <c r="AL10" s="14"/>
-      <c r="AM10" s="14"/>
-      <c r="AN10" s="14"/>
-      <c r="AO10" s="14"/>
-      <c r="AP10" s="14"/>
-      <c r="AQ10" s="14"/>
-      <c r="AR10" s="14"/>
-      <c r="AS10" s="14"/>
-      <c r="AT10" s="14"/>
-      <c r="AU10" s="14"/>
-      <c r="AV10" s="14"/>
-      <c r="AW10" s="14"/>
-      <c r="AX10" s="14"/>
-      <c r="AY10" s="14"/>
-      <c r="AZ10" s="14"/>
-      <c r="BA10" s="14"/>
-      <c r="BB10" s="14"/>
-      <c r="BC10" s="14"/>
-      <c r="BD10" s="14"/>
-      <c r="BE10" s="14"/>
-      <c r="BF10" s="14"/>
-      <c r="BG10" s="14"/>
-      <c r="BH10" s="14"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="12"/>
+      <c r="V10" s="12"/>
+      <c r="W10" s="12"/>
+      <c r="X10" s="12"/>
+      <c r="Y10" s="12"/>
+      <c r="Z10" s="12"/>
+      <c r="AA10" s="12"/>
+      <c r="AB10" s="12"/>
+      <c r="AC10" s="12"/>
+      <c r="AD10" s="12"/>
+      <c r="AE10" s="12"/>
+      <c r="AF10" s="12"/>
+      <c r="AG10" s="12"/>
+      <c r="AH10" s="12"/>
+      <c r="AI10" s="12"/>
+      <c r="AJ10" s="12"/>
+      <c r="AK10" s="12"/>
+      <c r="AL10" s="12"/>
+      <c r="AM10" s="12"/>
+      <c r="AN10" s="12"/>
+      <c r="AO10" s="12"/>
+      <c r="AP10" s="12"/>
+      <c r="AQ10" s="12"/>
+      <c r="AR10" s="12"/>
+      <c r="AS10" s="12"/>
+      <c r="AT10" s="12"/>
+      <c r="AU10" s="12"/>
+      <c r="AV10" s="12"/>
+      <c r="AW10" s="12"/>
+      <c r="AX10" s="12"/>
+      <c r="AY10" s="12"/>
+      <c r="AZ10" s="12"/>
+      <c r="BA10" s="12"/>
+      <c r="BB10" s="12"/>
+      <c r="BC10" s="12"/>
+      <c r="BD10" s="12"/>
+      <c r="BE10" s="12"/>
+      <c r="BF10" s="12"/>
+      <c r="BG10" s="12"/>
+      <c r="BH10" s="12"/>
     </row>
     <row r="11" s="3" customFormat="1" spans="2:60">
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="14"/>
-      <c r="O11" s="14"/>
-      <c r="P11" s="14"/>
-      <c r="Q11" s="14"/>
-      <c r="R11" s="14"/>
-      <c r="S11" s="14"/>
-      <c r="T11" s="14"/>
-      <c r="U11" s="14"/>
-      <c r="V11" s="14"/>
-      <c r="W11" s="14"/>
-      <c r="X11" s="14"/>
-      <c r="Y11" s="14"/>
-      <c r="Z11" s="14"/>
-      <c r="AA11" s="14"/>
-      <c r="AB11" s="14"/>
-      <c r="AC11" s="14"/>
-      <c r="AD11" s="14"/>
-      <c r="AE11" s="14"/>
-      <c r="AF11" s="14"/>
-      <c r="AG11" s="14"/>
-      <c r="AH11" s="14"/>
-      <c r="AI11" s="14"/>
-      <c r="AJ11" s="14"/>
-      <c r="AK11" s="14"/>
-      <c r="AL11" s="14"/>
-      <c r="AM11" s="14"/>
-      <c r="AN11" s="14"/>
-      <c r="AO11" s="14"/>
-      <c r="AP11" s="14"/>
-      <c r="AQ11" s="14"/>
-      <c r="AR11" s="14"/>
-      <c r="AS11" s="14"/>
-      <c r="AT11" s="14"/>
-      <c r="AU11" s="14"/>
-      <c r="AV11" s="14"/>
-      <c r="AW11" s="14"/>
-      <c r="AX11" s="14"/>
-      <c r="AY11" s="14"/>
-      <c r="AZ11" s="14"/>
-      <c r="BA11" s="14"/>
-      <c r="BB11" s="14"/>
-      <c r="BC11" s="14"/>
-      <c r="BD11" s="14"/>
-      <c r="BE11" s="14"/>
-      <c r="BF11" s="14"/>
-      <c r="BG11" s="14"/>
-      <c r="BH11" s="14"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="12"/>
+      <c r="V11" s="12"/>
+      <c r="W11" s="12"/>
+      <c r="X11" s="12"/>
+      <c r="Y11" s="12"/>
+      <c r="Z11" s="12"/>
+      <c r="AA11" s="12"/>
+      <c r="AB11" s="12"/>
+      <c r="AC11" s="12"/>
+      <c r="AD11" s="12"/>
+      <c r="AE11" s="12"/>
+      <c r="AF11" s="12"/>
+      <c r="AG11" s="12"/>
+      <c r="AH11" s="12"/>
+      <c r="AI11" s="12"/>
+      <c r="AJ11" s="12"/>
+      <c r="AK11" s="12"/>
+      <c r="AL11" s="12"/>
+      <c r="AM11" s="12"/>
+      <c r="AN11" s="12"/>
+      <c r="AO11" s="12"/>
+      <c r="AP11" s="12"/>
+      <c r="AQ11" s="12"/>
+      <c r="AR11" s="12"/>
+      <c r="AS11" s="12"/>
+      <c r="AT11" s="12"/>
+      <c r="AU11" s="12"/>
+      <c r="AV11" s="12"/>
+      <c r="AW11" s="12"/>
+      <c r="AX11" s="12"/>
+      <c r="AY11" s="12"/>
+      <c r="AZ11" s="12"/>
+      <c r="BA11" s="12"/>
+      <c r="BB11" s="12"/>
+      <c r="BC11" s="12"/>
+      <c r="BD11" s="12"/>
+      <c r="BE11" s="12"/>
+      <c r="BF11" s="12"/>
+      <c r="BG11" s="12"/>
+      <c r="BH11" s="12"/>
     </row>
     <row r="12" s="3" customFormat="1"/>
   </sheetData>

</xml_diff>